<commit_message>
removed duplicates that were data entry error
</commit_message>
<xml_diff>
--- a/Data/ESA_CBASS_metadata.xlsx
+++ b/Data/ESA_CBASS_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kira.turnham\Documents\GitHub\AS-CBASS.2026\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B724266-44D6-4CA7-87D9-1A35F8FFB7B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ADD23DB-EEFF-4EA1-BFC5-BDCCEE6C3E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6830F6C4-8395-44F5-9465-B5EF04B14AF4}"/>
+    <workbookView xWindow="7500" yWindow="1995" windowWidth="21600" windowHeight="11235" xr2:uid="{6830F6C4-8395-44F5-9465-B5EF04B14AF4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="20">
   <si>
     <t>AABR</t>
   </si>
@@ -511,7 +511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EABEA040-829B-4205-9B3F-8646AEB466BD}">
-  <dimension ref="A1:L170"/>
+  <dimension ref="A1:L167"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:12" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2906,34 +2906,34 @@
         <v>9</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F67" s="2">
-        <v>225</v>
+        <v>74</v>
       </c>
       <c r="G67" s="2">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="H67" s="2">
         <v>0</v>
       </c>
       <c r="I67" s="2">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="J67" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K67" s="1"/>
+      <c r="K67" s="6"/>
       <c r="L67" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="68" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B68" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C68" s="2">
         <v>20260216</v>
@@ -2942,34 +2942,34 @@
         <v>9</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F68" s="2">
-        <v>105</v>
+        <v>67</v>
       </c>
       <c r="G68" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H68" s="2">
         <v>0</v>
       </c>
       <c r="I68" s="2">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="J68" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K68" s="1"/>
+      <c r="K68" s="6"/>
       <c r="L68" s="2">
-        <v>7</v>
+        <v>16</v>
       </c>
     </row>
     <row r="69" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B69" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C69" s="2">
         <v>20260216</v>
@@ -2981,23 +2981,23 @@
         <v>7</v>
       </c>
       <c r="F69" s="2">
-        <v>74</v>
+        <v>45</v>
       </c>
       <c r="G69" s="2">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="H69" s="2">
         <v>0</v>
       </c>
       <c r="I69" s="2">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J69" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K69" s="6"/>
       <c r="L69" s="2">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="70" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3017,7 +3017,7 @@
         <v>7</v>
       </c>
       <c r="F70" s="2">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="G70" s="2">
         <v>1</v>
@@ -3026,14 +3026,14 @@
         <v>0</v>
       </c>
       <c r="I70" s="2">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="J70" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K70" s="6"/>
       <c r="L70" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="71" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3050,34 +3050,34 @@
         <v>9</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F71" s="2">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="G71" s="2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H71" s="2">
         <v>0</v>
       </c>
       <c r="I71" s="2">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="J71" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K71" s="6"/>
       <c r="L71" s="2">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="72" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B72" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C72" s="2">
         <v>20260216</v>
@@ -3089,31 +3089,33 @@
         <v>7</v>
       </c>
       <c r="F72" s="2">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G72" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H72" s="2">
         <v>0</v>
       </c>
       <c r="I72" s="2">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="J72" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K72" s="6"/>
+      <c r="K72" s="8">
+        <v>21</v>
+      </c>
       <c r="L72" s="2">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="73" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B73" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C73" s="2">
         <v>20260216</v>
@@ -3122,26 +3124,28 @@
         <v>9</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F73" s="2">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="G73" s="2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H73" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I73" s="2">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="J73" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K73" s="6"/>
+      <c r="K73" s="8">
+        <v>24</v>
+      </c>
       <c r="L73" s="2">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="74" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3161,25 +3165,25 @@
         <v>7</v>
       </c>
       <c r="F74" s="2">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="G74" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H74" s="2">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I74" s="2">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="J74" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K74" s="8">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="L74" s="2">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="75" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3199,10 +3203,10 @@
         <v>7</v>
       </c>
       <c r="F75" s="2">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="G75" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H75" s="2">
         <v>10</v>
@@ -3213,11 +3217,9 @@
       <c r="J75" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K75" s="8">
+      <c r="K75" s="6"/>
+      <c r="L75" s="2">
         <v>24</v>
-      </c>
-      <c r="L75" s="2">
-        <v>22</v>
       </c>
     </row>
     <row r="76" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3237,33 +3239,31 @@
         <v>7</v>
       </c>
       <c r="F76" s="2">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="G76" s="2">
         <v>0</v>
       </c>
       <c r="H76" s="2">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I76" s="2">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="J76" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K76" s="8">
-        <v>23</v>
-      </c>
+      <c r="K76" s="6"/>
       <c r="L76" s="2">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="77" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B77" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C77" s="2">
         <v>20260216</v>
@@ -3272,34 +3272,34 @@
         <v>9</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F77" s="2">
+        <v>47</v>
+      </c>
+      <c r="G77" s="2">
+        <v>0</v>
+      </c>
+      <c r="H77" s="2">
+        <v>0</v>
+      </c>
+      <c r="I77" s="2">
         <v>39</v>
-      </c>
-      <c r="G77" s="2">
-        <v>0</v>
-      </c>
-      <c r="H77" s="2">
-        <v>10</v>
-      </c>
-      <c r="I77" s="2">
-        <v>30</v>
       </c>
       <c r="J77" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K77" s="6"/>
       <c r="L77" s="2">
-        <v>24</v>
+        <v>31</v>
       </c>
     </row>
     <row r="78" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B78" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C78" s="2">
         <v>20260216</v>
@@ -3308,10 +3308,10 @@
         <v>9</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F78" s="2">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="G78" s="2">
         <v>0</v>
@@ -3320,22 +3320,22 @@
         <v>0</v>
       </c>
       <c r="I78" s="2">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="J78" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K78" s="6"/>
       <c r="L78" s="2">
-        <v>25</v>
+        <v>32</v>
       </c>
     </row>
     <row r="79" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B79" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C79" s="2">
         <v>20260216</v>
@@ -3344,26 +3344,26 @@
         <v>9</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F79" s="2">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G79" s="2">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="H79" s="2">
         <v>0</v>
       </c>
       <c r="I79" s="2">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J79" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K79" s="1"/>
+      <c r="K79" s="6"/>
       <c r="L79" s="2">
-        <v>8</v>
+        <v>33</v>
       </c>
     </row>
     <row r="80" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3383,23 +3383,23 @@
         <v>9</v>
       </c>
       <c r="F80" s="2">
-        <v>47</v>
+        <v>125</v>
       </c>
       <c r="G80" s="2">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H80" s="2">
         <v>0</v>
       </c>
       <c r="I80" s="2">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="J80" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K80" s="6"/>
       <c r="L80" s="2">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="81" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3419,7 +3419,7 @@
         <v>9</v>
       </c>
       <c r="F81" s="2">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="G81" s="2">
         <v>0</v>
@@ -3428,22 +3428,22 @@
         <v>0</v>
       </c>
       <c r="I81" s="2">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="J81" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K81" s="6"/>
       <c r="L81" s="2">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="82" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B82" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C82" s="2">
         <v>20260216</v>
@@ -3452,26 +3452,26 @@
         <v>9</v>
       </c>
       <c r="E82" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F82" s="2">
+        <v>53</v>
+      </c>
+      <c r="G82" s="2">
+        <v>5</v>
+      </c>
+      <c r="H82" s="2">
+        <v>0</v>
+      </c>
+      <c r="I82" s="2">
+        <v>33</v>
+      </c>
+      <c r="J82" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K82" s="1"/>
+      <c r="L82" s="2">
         <v>9</v>
-      </c>
-      <c r="F82" s="2">
-        <v>80</v>
-      </c>
-      <c r="G82" s="2">
-        <v>0</v>
-      </c>
-      <c r="H82" s="2">
-        <v>0</v>
-      </c>
-      <c r="I82" s="2">
-        <v>38</v>
-      </c>
-      <c r="J82" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="K82" s="6"/>
-      <c r="L82" s="2">
-        <v>33</v>
       </c>
     </row>
     <row r="83" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3479,7 +3479,7 @@
         <v>10</v>
       </c>
       <c r="B83" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C83" s="2">
         <v>20260216</v>
@@ -3488,26 +3488,28 @@
         <v>9</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F83" s="2">
-        <v>125</v>
+        <v>64</v>
       </c>
       <c r="G83" s="2">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H83" s="2">
         <v>0</v>
       </c>
       <c r="I83" s="2">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="J83" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K83" s="6"/>
+      <c r="K83" s="2">
+        <v>31</v>
+      </c>
       <c r="L83" s="2">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="84" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3515,7 +3517,7 @@
         <v>10</v>
       </c>
       <c r="B84" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C84" s="2">
         <v>20260216</v>
@@ -3524,34 +3526,34 @@
         <v>9</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F84" s="2">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="G84" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H84" s="2">
         <v>0</v>
       </c>
       <c r="I84" s="2">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="J84" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K84" s="6"/>
+      <c r="K84" s="1"/>
       <c r="L84" s="2">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="85" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B85" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C85" s="2">
         <v>20260216</v>
@@ -3563,7 +3565,7 @@
         <v>11</v>
       </c>
       <c r="F85" s="2">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="G85" s="2">
         <v>5</v>
@@ -3572,14 +3574,14 @@
         <v>0</v>
       </c>
       <c r="I85" s="2">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J85" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K85" s="1"/>
       <c r="L85" s="2">
-        <v>9</v>
+        <v>38</v>
       </c>
     </row>
     <row r="86" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3599,25 +3601,23 @@
         <v>11</v>
       </c>
       <c r="F86" s="2">
-        <v>64</v>
+        <v>31</v>
       </c>
       <c r="G86" s="2">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H86" s="2">
         <v>0</v>
       </c>
       <c r="I86" s="2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J86" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K86" s="2">
-        <v>31</v>
-      </c>
+      <c r="K86" s="1"/>
       <c r="L86" s="2">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="87" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3628,32 +3628,32 @@
         <v>3</v>
       </c>
       <c r="C87" s="2">
-        <v>20260216</v>
+        <v>20260217</v>
       </c>
       <c r="D87" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F87" s="2">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="G87" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H87" s="2">
         <v>0</v>
       </c>
       <c r="I87" s="2">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J87" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K87" s="1"/>
+      <c r="K87" s="6"/>
       <c r="L87" s="2">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="88" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3664,76 +3664,76 @@
         <v>3</v>
       </c>
       <c r="C88" s="2">
-        <v>20260216</v>
+        <v>20260217</v>
       </c>
       <c r="D88" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F88" s="2">
-        <v>62</v>
+        <v>94</v>
       </c>
       <c r="G88" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H88" s="2">
         <v>0</v>
       </c>
       <c r="I88" s="2">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="J88" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K88" s="1"/>
+      <c r="K88" s="6"/>
       <c r="L88" s="2">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="89" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B89" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C89" s="2">
-        <v>20260216</v>
+        <v>20260217</v>
       </c>
       <c r="D89" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F89" s="2">
-        <v>31</v>
+        <v>73</v>
       </c>
       <c r="G89" s="2">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H89" s="2">
         <v>0</v>
       </c>
       <c r="I89" s="2">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J89" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K89" s="1"/>
+      <c r="K89" s="6"/>
       <c r="L89" s="2">
-        <v>39</v>
+        <v>21</v>
       </c>
     </row>
     <row r="90" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B90" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C90" s="2">
         <v>20260217</v>
@@ -3742,34 +3742,34 @@
         <v>10</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F90" s="2">
-        <v>140</v>
+        <v>42</v>
       </c>
       <c r="G90" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H90" s="2">
         <v>0</v>
       </c>
       <c r="I90" s="2">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J90" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K90" s="6"/>
       <c r="L90" s="2">
-        <v>31</v>
+        <v>22</v>
       </c>
     </row>
     <row r="91" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B91" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C91" s="2">
         <v>20260217</v>
@@ -3778,34 +3778,34 @@
         <v>10</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F91" s="2">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="G91" s="2">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H91" s="2">
         <v>0</v>
       </c>
       <c r="I91" s="2">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J91" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K91" s="6"/>
       <c r="L91" s="2">
-        <v>32</v>
+        <v>11</v>
       </c>
     </row>
     <row r="92" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B92" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C92" s="2">
         <v>20260217</v>
@@ -3817,31 +3817,31 @@
         <v>7</v>
       </c>
       <c r="F92" s="2">
-        <v>73</v>
+        <v>29</v>
       </c>
       <c r="G92" s="2">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H92" s="2">
         <v>0</v>
       </c>
       <c r="I92" s="2">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="J92" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K92" s="6"/>
       <c r="L92" s="2">
-        <v>21</v>
+        <v>12</v>
       </c>
     </row>
     <row r="93" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B93" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C93" s="2">
         <v>20260217</v>
@@ -3853,23 +3853,23 @@
         <v>7</v>
       </c>
       <c r="F93" s="2">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="G93" s="2">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H93" s="2">
         <v>0</v>
       </c>
       <c r="I93" s="2">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="J93" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K93" s="6"/>
       <c r="L93" s="2">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="94" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3889,31 +3889,31 @@
         <v>7</v>
       </c>
       <c r="F94" s="2">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="G94" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H94" s="2">
         <v>0</v>
       </c>
       <c r="I94" s="2">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J94" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K94" s="6"/>
       <c r="L94" s="2">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="95" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B95" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C95" s="2">
         <v>20260217</v>
@@ -3922,34 +3922,34 @@
         <v>10</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F95" s="2">
+        <v>81</v>
+      </c>
+      <c r="G95" s="2">
+        <v>0</v>
+      </c>
+      <c r="H95" s="2">
+        <v>0</v>
+      </c>
+      <c r="I95" s="2">
         <v>29</v>
-      </c>
-      <c r="G95" s="2">
-        <v>0</v>
-      </c>
-      <c r="H95" s="2">
-        <v>0</v>
-      </c>
-      <c r="I95" s="2">
-        <v>35</v>
       </c>
       <c r="J95" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K95" s="6"/>
       <c r="L95" s="2">
-        <v>12</v>
+        <v>33</v>
       </c>
     </row>
     <row r="96" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B96" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C96" s="2">
         <v>20260217</v>
@@ -3958,34 +3958,34 @@
         <v>10</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F96" s="2">
-        <v>21</v>
+        <v>142</v>
       </c>
       <c r="G96" s="2">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H96" s="2">
         <v>0</v>
       </c>
       <c r="I96" s="2">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="J96" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K96" s="6"/>
       <c r="L96" s="2">
-        <v>13</v>
+        <v>35</v>
       </c>
     </row>
     <row r="97" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B97" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C97" s="2">
         <v>20260217</v>
@@ -3994,34 +3994,34 @@
         <v>10</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F97" s="2">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="G97" s="2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H97" s="2">
         <v>0</v>
       </c>
       <c r="I97" s="2">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="J97" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K97" s="6"/>
       <c r="L97" s="2">
-        <v>14</v>
+        <v>23</v>
       </c>
     </row>
     <row r="98" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B98" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C98" s="2">
         <v>20260217</v>
@@ -4030,34 +4030,34 @@
         <v>10</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F98" s="2">
-        <v>81</v>
+        <v>32</v>
       </c>
       <c r="G98" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H98" s="2">
         <v>0</v>
       </c>
       <c r="I98" s="2">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="J98" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K98" s="6"/>
       <c r="L98" s="2">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="99" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B99" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C99" s="2">
         <v>20260217</v>
@@ -4066,34 +4066,34 @@
         <v>10</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F99" s="2">
-        <v>142</v>
+        <v>40</v>
       </c>
       <c r="G99" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H99" s="2">
         <v>0</v>
       </c>
       <c r="I99" s="2">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="J99" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K99" s="6"/>
       <c r="L99" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="100" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B100" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C100" s="2">
         <v>20260217</v>
@@ -4105,31 +4105,31 @@
         <v>11</v>
       </c>
       <c r="F100" s="2">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="G100" s="2">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="H100" s="2">
         <v>0</v>
       </c>
       <c r="I100" s="2">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="J100" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K100" s="6"/>
       <c r="L100" s="2">
-        <v>23</v>
+        <v>37</v>
       </c>
     </row>
     <row r="101" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B101" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C101" s="2">
         <v>20260217</v>
@@ -4141,23 +4141,23 @@
         <v>11</v>
       </c>
       <c r="F101" s="2">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="G101" s="2">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H101" s="2">
         <v>0</v>
       </c>
       <c r="I101" s="2">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="J101" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K101" s="6"/>
       <c r="L101" s="2">
-        <v>24</v>
+        <v>38</v>
       </c>
     </row>
     <row r="102" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4177,31 +4177,31 @@
         <v>11</v>
       </c>
       <c r="F102" s="2">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="G102" s="2">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H102" s="2">
         <v>0</v>
       </c>
       <c r="I102" s="2">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="J102" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K102" s="6"/>
       <c r="L102" s="2">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="103" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B103" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C103" s="2">
         <v>20260217</v>
@@ -4213,31 +4213,31 @@
         <v>11</v>
       </c>
       <c r="F103" s="2">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="G103" s="2">
-        <v>65</v>
+        <v>3</v>
       </c>
       <c r="H103" s="2">
         <v>0</v>
       </c>
       <c r="I103" s="2">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="J103" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K103" s="6"/>
       <c r="L103" s="2">
-        <v>37</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B104" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C104" s="2">
         <v>20260217</v>
@@ -4249,31 +4249,31 @@
         <v>11</v>
       </c>
       <c r="F104" s="2">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="G104" s="2">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H104" s="2">
         <v>0</v>
       </c>
       <c r="I104" s="2">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J104" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K104" s="6"/>
       <c r="L104" s="2">
-        <v>38</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B105" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C105" s="2">
         <v>20260217</v>
@@ -4285,10 +4285,10 @@
         <v>11</v>
       </c>
       <c r="F105" s="2">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="G105" s="2">
-        <v>10</v>
+        <v>75</v>
       </c>
       <c r="H105" s="2">
         <v>0</v>
@@ -4301,7 +4301,7 @@
       </c>
       <c r="K105" s="6"/>
       <c r="L105" s="2">
-        <v>39</v>
+        <v>5</v>
       </c>
     </row>
     <row r="106" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4321,23 +4321,23 @@
         <v>11</v>
       </c>
       <c r="F106" s="2">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G106" s="2">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="H106" s="2">
         <v>0</v>
       </c>
       <c r="I106" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J106" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K106" s="6"/>
       <c r="L106" s="2">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="107" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4348,32 +4348,32 @@
         <v>3</v>
       </c>
       <c r="C107" s="2">
-        <v>20260217</v>
+        <v>20260219</v>
       </c>
       <c r="D107" s="1">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F107" s="2">
-        <v>45</v>
+        <v>73</v>
       </c>
       <c r="G107" s="2">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H107" s="2">
         <v>0</v>
       </c>
       <c r="I107" s="2">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="J107" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K107" s="6"/>
       <c r="L107" s="2">
-        <v>3</v>
+        <v>26</v>
       </c>
     </row>
     <row r="108" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4384,76 +4384,76 @@
         <v>3</v>
       </c>
       <c r="C108" s="2">
-        <v>20260217</v>
+        <v>20260219</v>
       </c>
       <c r="D108" s="1">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F108" s="2">
-        <v>67</v>
+        <v>127</v>
       </c>
       <c r="G108" s="2">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="H108" s="2">
         <v>0</v>
       </c>
       <c r="I108" s="2">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="J108" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K108" s="6"/>
       <c r="L108" s="2">
-        <v>5</v>
+        <v>27</v>
       </c>
     </row>
     <row r="109" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B109" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C109" s="2">
-        <v>20260217</v>
+        <v>20260219</v>
       </c>
       <c r="D109" s="1">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F109" s="2">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="G109" s="2">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="H109" s="2">
         <v>0</v>
       </c>
       <c r="I109" s="2">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="J109" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K109" s="6"/>
       <c r="L109" s="2">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="110" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B110" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C110" s="2">
         <v>20260219</v>
@@ -4462,10 +4462,10 @@
         <v>3</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F110" s="2">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="G110" s="2">
         <v>0</v>
@@ -4474,22 +4474,22 @@
         <v>0</v>
       </c>
       <c r="I110" s="2">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="J110" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K110" s="6"/>
       <c r="L110" s="2">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
     <row r="111" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B111" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C111" s="2">
         <v>20260219</v>
@@ -4498,26 +4498,26 @@
         <v>3</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F111" s="2">
-        <v>127</v>
+        <v>45</v>
       </c>
       <c r="G111" s="2">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H111" s="2">
         <v>0</v>
       </c>
       <c r="I111" s="2">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="J111" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K111" s="6"/>
       <c r="L111" s="2">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
     <row r="112" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4537,31 +4537,31 @@
         <v>7</v>
       </c>
       <c r="F112" s="2">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="G112" s="2">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="H112" s="2">
         <v>0</v>
       </c>
       <c r="I112" s="2">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="J112" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K112" s="6"/>
       <c r="L112" s="2">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="113" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B113" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C113" s="2">
         <v>20260219</v>
@@ -4573,31 +4573,31 @@
         <v>7</v>
       </c>
       <c r="F113" s="2">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="G113" s="2">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H113" s="2">
         <v>0</v>
       </c>
       <c r="I113" s="2">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="J113" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K113" s="6"/>
       <c r="L113" s="2">
-        <v>14</v>
+        <v>36</v>
       </c>
     </row>
     <row r="114" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B114" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C114" s="2">
         <v>20260219</v>
@@ -4609,31 +4609,31 @@
         <v>7</v>
       </c>
       <c r="F114" s="2">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="G114" s="2">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="H114" s="2">
         <v>0</v>
       </c>
       <c r="I114" s="2">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J114" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K114" s="6"/>
       <c r="L114" s="2">
-        <v>15</v>
+        <v>38</v>
       </c>
     </row>
     <row r="115" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B115" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C115" s="2">
         <v>20260219</v>
@@ -4645,23 +4645,23 @@
         <v>7</v>
       </c>
       <c r="F115" s="2">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="G115" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H115" s="2">
         <v>0</v>
       </c>
       <c r="I115" s="2">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="J115" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K115" s="6"/>
       <c r="L115" s="2">
-        <v>16</v>
+        <v>39</v>
       </c>
     </row>
     <row r="116" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4681,23 +4681,23 @@
         <v>7</v>
       </c>
       <c r="F116" s="2">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="G116" s="2">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="H116" s="2">
         <v>0</v>
       </c>
       <c r="I116" s="2">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="J116" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K116" s="6"/>
       <c r="L116" s="2">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="117" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4714,26 +4714,26 @@
         <v>3</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F117" s="2">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="G117" s="2">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="H117" s="2">
         <v>0</v>
       </c>
       <c r="I117" s="2">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J117" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K117" s="6"/>
       <c r="L117" s="2">
-        <v>38</v>
+        <v>29</v>
       </c>
     </row>
     <row r="118" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4750,34 +4750,34 @@
         <v>3</v>
       </c>
       <c r="E118" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F118" s="2">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="G118" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H118" s="2">
         <v>0</v>
       </c>
       <c r="I118" s="2">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="J118" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K118" s="6"/>
       <c r="L118" s="2">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="119" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B119" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C119" s="2">
         <v>20260219</v>
@@ -4786,34 +4786,34 @@
         <v>3</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F119" s="2">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G119" s="2">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="H119" s="2">
         <v>0</v>
       </c>
       <c r="I119" s="2">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J119" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K119" s="6"/>
       <c r="L119" s="2">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="120" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B120" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C120" s="2">
         <v>20260219</v>
@@ -4822,34 +4822,34 @@
         <v>3</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F120" s="2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G120" s="2">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="H120" s="2">
         <v>0</v>
       </c>
       <c r="I120" s="2">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="J120" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K120" s="6"/>
       <c r="L120" s="2">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="121" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B121" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C121" s="2">
         <v>20260219</v>
@@ -4858,26 +4858,26 @@
         <v>3</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F121" s="2">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="G121" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H121" s="2">
         <v>0</v>
       </c>
       <c r="I121" s="2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J121" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K121" s="6"/>
       <c r="L121" s="2">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="122" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4897,31 +4897,31 @@
         <v>11</v>
       </c>
       <c r="F122" s="2">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="G122" s="2">
-        <v>70</v>
+        <v>2</v>
       </c>
       <c r="H122" s="2">
         <v>0</v>
       </c>
       <c r="I122" s="2">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="J122" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K122" s="6"/>
       <c r="L122" s="2">
-        <v>33</v>
+        <v>66</v>
       </c>
     </row>
     <row r="123" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B123" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C123" s="2">
         <v>20260219</v>
@@ -4933,31 +4933,31 @@
         <v>11</v>
       </c>
       <c r="F123" s="2">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="G123" s="2">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="H123" s="2">
         <v>0</v>
       </c>
       <c r="I123" s="2">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="J123" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K123" s="6"/>
       <c r="L123" s="2">
-        <v>34</v>
+        <v>61</v>
       </c>
     </row>
     <row r="124" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B124" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C124" s="2">
         <v>20260219</v>
@@ -4969,31 +4969,31 @@
         <v>11</v>
       </c>
       <c r="F124" s="2">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="G124" s="2">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="H124" s="2">
         <v>0</v>
       </c>
       <c r="I124" s="2">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="J124" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K124" s="6"/>
       <c r="L124" s="2">
-        <v>35</v>
+        <v>62</v>
       </c>
     </row>
     <row r="125" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B125" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C125" s="2">
         <v>20260219</v>
@@ -5005,23 +5005,23 @@
         <v>11</v>
       </c>
       <c r="F125" s="2">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="G125" s="2">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="H125" s="2">
         <v>0</v>
       </c>
       <c r="I125" s="2">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="J125" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K125" s="6"/>
       <c r="L125" s="2">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="126" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5041,23 +5041,23 @@
         <v>11</v>
       </c>
       <c r="F126" s="2">
-        <v>40</v>
+        <v>82</v>
       </c>
       <c r="G126" s="2">
-        <v>5</v>
+        <v>70</v>
       </c>
       <c r="H126" s="2">
         <v>0</v>
       </c>
       <c r="I126" s="2">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="J126" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K126" s="6"/>
       <c r="L126" s="2">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="127" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5068,19 +5068,19 @@
         <v>2</v>
       </c>
       <c r="C127" s="2">
-        <v>20260219</v>
+        <v>20260220</v>
       </c>
       <c r="D127" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E127" s="1" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F127" s="2">
-        <v>43</v>
+        <v>160</v>
       </c>
       <c r="G127" s="2">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="H127" s="2">
         <v>0</v>
@@ -5093,7 +5093,7 @@
       </c>
       <c r="K127" s="6"/>
       <c r="L127" s="2">
-        <v>62</v>
+        <v>6</v>
       </c>
     </row>
     <row r="128" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5104,76 +5104,76 @@
         <v>2</v>
       </c>
       <c r="C128" s="2">
-        <v>20260219</v>
+        <v>20260220</v>
       </c>
       <c r="D128" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E128" s="1" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F128" s="2">
-        <v>47</v>
+        <v>205</v>
       </c>
       <c r="G128" s="2">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H128" s="2">
         <v>0</v>
       </c>
       <c r="I128" s="2">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="J128" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K128" s="6"/>
       <c r="L128" s="2">
-        <v>63</v>
+        <v>7</v>
       </c>
     </row>
     <row r="129" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B129" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C129" s="2">
-        <v>20260219</v>
+        <v>20260220</v>
       </c>
       <c r="D129" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E129" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F129" s="2">
-        <v>82</v>
+        <v>52</v>
       </c>
       <c r="G129" s="2">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="H129" s="2">
         <v>0</v>
       </c>
       <c r="I129" s="2">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="J129" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K129" s="6"/>
       <c r="L129" s="2">
-        <v>64</v>
+        <v>24</v>
       </c>
     </row>
     <row r="130" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B130" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C130" s="2">
         <v>20260220</v>
@@ -5182,34 +5182,34 @@
         <v>4</v>
       </c>
       <c r="E130" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F130" s="2">
-        <v>160</v>
+        <v>45</v>
       </c>
       <c r="G130" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H130" s="2">
         <v>0</v>
       </c>
       <c r="I130" s="2">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="J130" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K130" s="6"/>
       <c r="L130" s="2">
-        <v>6</v>
+        <v>25</v>
       </c>
     </row>
     <row r="131" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B131" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C131" s="2">
         <v>20260220</v>
@@ -5218,26 +5218,26 @@
         <v>4</v>
       </c>
       <c r="E131" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F131" s="2">
-        <v>205</v>
+        <v>35</v>
       </c>
       <c r="G131" s="2">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="H131" s="2">
         <v>0</v>
       </c>
       <c r="I131" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J131" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K131" s="6"/>
       <c r="L131" s="2">
-        <v>7</v>
+        <v>21</v>
       </c>
     </row>
     <row r="132" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5257,31 +5257,31 @@
         <v>7</v>
       </c>
       <c r="F132" s="2">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="G132" s="2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H132" s="2">
         <v>0</v>
       </c>
       <c r="I132" s="2">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J132" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K132" s="6"/>
       <c r="L132" s="2">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="133" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B133" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C133" s="2">
         <v>20260220</v>
@@ -5293,7 +5293,7 @@
         <v>7</v>
       </c>
       <c r="F133" s="2">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="G133" s="2">
         <v>0</v>
@@ -5302,22 +5302,24 @@
         <v>0</v>
       </c>
       <c r="I133" s="2">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J133" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K133" s="6"/>
+      <c r="K133" s="8">
+        <v>10</v>
+      </c>
       <c r="L133" s="2">
-        <v>25</v>
+        <v>33</v>
       </c>
     </row>
     <row r="134" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B134" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C134" s="2">
         <v>20260220</v>
@@ -5329,31 +5331,31 @@
         <v>7</v>
       </c>
       <c r="F134" s="2">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G134" s="2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H134" s="2">
         <v>0</v>
       </c>
       <c r="I134" s="2">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J134" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K134" s="6"/>
       <c r="L134" s="2">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="135" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B135" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C135" s="2">
         <v>20260220</v>
@@ -5365,10 +5367,10 @@
         <v>7</v>
       </c>
       <c r="F135" s="2">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="G135" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H135" s="2">
         <v>0</v>
@@ -5381,7 +5383,7 @@
       </c>
       <c r="K135" s="6"/>
       <c r="L135" s="2">
-        <v>22</v>
+        <v>35</v>
       </c>
     </row>
     <row r="136" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5401,25 +5403,23 @@
         <v>7</v>
       </c>
       <c r="F136" s="2">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G136" s="2">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H136" s="2">
         <v>0</v>
       </c>
       <c r="I136" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J136" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="K136" s="8">
-        <v>10</v>
-      </c>
+      <c r="K136" s="6"/>
       <c r="L136" s="2">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="137" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5439,31 +5439,31 @@
         <v>7</v>
       </c>
       <c r="F137" s="2">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="G137" s="2">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H137" s="2">
         <v>0</v>
       </c>
       <c r="I137" s="2">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J137" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K137" s="6"/>
       <c r="L137" s="2">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="138" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B138" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C138" s="2">
         <v>20260220</v>
@@ -5472,34 +5472,34 @@
         <v>4</v>
       </c>
       <c r="E138" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F138" s="2">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="G138" s="2">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H138" s="2">
         <v>0</v>
       </c>
       <c r="I138" s="2">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J138" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K138" s="6"/>
       <c r="L138" s="2">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="139" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B139" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C139" s="2">
         <v>20260220</v>
@@ -5508,34 +5508,34 @@
         <v>4</v>
       </c>
       <c r="E139" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F139" s="2">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="G139" s="2">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="H139" s="2">
         <v>0</v>
       </c>
       <c r="I139" s="2">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J139" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K139" s="6"/>
       <c r="L139" s="2">
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="140" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B140" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C140" s="2">
         <v>20260220</v>
@@ -5544,26 +5544,26 @@
         <v>4</v>
       </c>
       <c r="E140" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F140" s="2">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G140" s="2">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="H140" s="2">
         <v>0</v>
       </c>
       <c r="I140" s="2">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J140" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K140" s="6"/>
       <c r="L140" s="2">
-        <v>27</v>
+        <v>41</v>
       </c>
     </row>
     <row r="141" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5580,26 +5580,26 @@
         <v>4</v>
       </c>
       <c r="E141" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F141" s="2">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="G141" s="2">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H141" s="2">
         <v>0</v>
       </c>
       <c r="I141" s="2">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="J141" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K141" s="6"/>
       <c r="L141" s="2">
-        <v>10</v>
+        <v>42</v>
       </c>
     </row>
     <row r="142" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5616,26 +5616,26 @@
         <v>4</v>
       </c>
       <c r="E142" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F142" s="2">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="G142" s="2">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="H142" s="2">
         <v>0</v>
       </c>
       <c r="I142" s="2">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J142" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K142" s="6"/>
       <c r="L142" s="2">
-        <v>16</v>
+        <v>43</v>
       </c>
     </row>
     <row r="143" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5655,10 +5655,10 @@
         <v>11</v>
       </c>
       <c r="F143" s="2">
-        <v>43</v>
+        <v>90</v>
       </c>
       <c r="G143" s="2">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H143" s="2">
         <v>0</v>
@@ -5671,15 +5671,15 @@
       </c>
       <c r="K143" s="6"/>
       <c r="L143" s="2">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="144" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B144" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C144" s="2">
         <v>20260220</v>
@@ -5691,31 +5691,31 @@
         <v>11</v>
       </c>
       <c r="F144" s="2">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="G144" s="2">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="H144" s="2">
         <v>0</v>
       </c>
       <c r="I144" s="2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J144" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K144" s="6"/>
       <c r="L144" s="2">
-        <v>42</v>
+        <v>61</v>
       </c>
     </row>
     <row r="145" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B145" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C145" s="2">
         <v>20260220</v>
@@ -5727,31 +5727,31 @@
         <v>11</v>
       </c>
       <c r="F145" s="2">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="G145" s="2">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="H145" s="2">
         <v>0</v>
       </c>
       <c r="I145" s="2">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="J145" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K145" s="6"/>
       <c r="L145" s="2">
-        <v>43</v>
+        <v>62</v>
       </c>
     </row>
     <row r="146" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B146" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C146" s="2">
         <v>20260220</v>
@@ -5763,23 +5763,23 @@
         <v>11</v>
       </c>
       <c r="F146" s="2">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="G146" s="2">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="H146" s="2">
         <v>0</v>
       </c>
       <c r="I146" s="2">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J146" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K146" s="6"/>
       <c r="L146" s="2">
-        <v>44</v>
+        <v>64</v>
       </c>
     </row>
     <row r="147" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5802,128 +5802,128 @@
         <v>38</v>
       </c>
       <c r="G147" s="2">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="H147" s="2">
         <v>0</v>
       </c>
       <c r="I147" s="2">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J147" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K147" s="6"/>
       <c r="L147" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="148" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B148" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C148" s="2">
-        <v>20260220</v>
+        <v>20260223</v>
       </c>
       <c r="D148" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E148" s="1" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F148" s="2">
-        <v>30</v>
+        <v>420</v>
       </c>
       <c r="G148" s="2">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="H148" s="2">
         <v>0</v>
       </c>
       <c r="I148" s="2">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="J148" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K148" s="6"/>
       <c r="L148" s="2">
-        <v>62</v>
+        <v>33</v>
       </c>
     </row>
     <row r="149" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B149" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C149" s="2">
-        <v>20260220</v>
+        <v>20260223</v>
       </c>
       <c r="D149" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E149" s="1" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F149" s="2">
-        <v>60</v>
+        <v>145</v>
       </c>
       <c r="G149" s="2">
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="H149" s="2">
         <v>0</v>
       </c>
       <c r="I149" s="2">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J149" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K149" s="6"/>
       <c r="L149" s="2">
-        <v>64</v>
+        <v>34</v>
       </c>
     </row>
     <row r="150" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B150" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C150" s="2">
-        <v>20260220</v>
+        <v>20260223</v>
       </c>
       <c r="D150" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E150" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F150" s="2">
+        <v>115</v>
+      </c>
+      <c r="G150" s="2">
+        <v>15</v>
+      </c>
+      <c r="H150" s="2">
+        <v>0</v>
+      </c>
+      <c r="I150" s="2">
         <v>38</v>
-      </c>
-      <c r="G150" s="2">
-        <v>25</v>
-      </c>
-      <c r="H150" s="2">
-        <v>0</v>
-      </c>
-      <c r="I150" s="2">
-        <v>39</v>
       </c>
       <c r="J150" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K150" s="6"/>
       <c r="L150" s="2">
-        <v>63</v>
+        <v>35</v>
       </c>
     </row>
     <row r="151" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5940,13 +5940,13 @@
         <v>5</v>
       </c>
       <c r="E151" s="1" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F151" s="2">
-        <v>420</v>
+        <v>54</v>
       </c>
       <c r="G151" s="2">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="H151" s="2">
         <v>0</v>
@@ -5959,15 +5959,15 @@
       </c>
       <c r="K151" s="6"/>
       <c r="L151" s="2">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="152" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B152" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C152" s="2">
         <v>20260223</v>
@@ -5976,34 +5976,34 @@
         <v>5</v>
       </c>
       <c r="E152" s="1" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F152" s="2">
-        <v>145</v>
+        <v>45</v>
       </c>
       <c r="G152" s="2">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H152" s="2">
         <v>0</v>
       </c>
       <c r="I152" s="2">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="J152" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K152" s="6"/>
       <c r="L152" s="2">
-        <v>34</v>
+        <v>41</v>
       </c>
     </row>
     <row r="153" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B153" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C153" s="2">
         <v>20260223</v>
@@ -6012,34 +6012,34 @@
         <v>5</v>
       </c>
       <c r="E153" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F153" s="2">
-        <v>115</v>
+        <v>64</v>
       </c>
       <c r="G153" s="2">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="H153" s="2">
         <v>0</v>
       </c>
       <c r="I153" s="2">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J153" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K153" s="6"/>
       <c r="L153" s="2">
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="154" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B154" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C154" s="2">
         <v>20260223</v>
@@ -6048,26 +6048,26 @@
         <v>5</v>
       </c>
       <c r="E154" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F154" s="2">
-        <v>54</v>
+        <v>125</v>
       </c>
       <c r="G154" s="2">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="H154" s="2">
         <v>0</v>
       </c>
       <c r="I154" s="2">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="J154" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K154" s="6"/>
       <c r="L154" s="2">
-        <v>26</v>
+        <v>43</v>
       </c>
     </row>
     <row r="155" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6087,31 +6087,31 @@
         <v>11</v>
       </c>
       <c r="F155" s="2">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="G155" s="2">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="H155" s="2">
         <v>0</v>
       </c>
       <c r="I155" s="2">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="J155" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K155" s="6"/>
       <c r="L155" s="2">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="156" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B156" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C156" s="2">
         <v>20260223</v>
@@ -6123,31 +6123,31 @@
         <v>11</v>
       </c>
       <c r="F156" s="2">
-        <v>64</v>
+        <v>98</v>
       </c>
       <c r="G156" s="2">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="H156" s="2">
         <v>0</v>
       </c>
       <c r="I156" s="2">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="J156" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K156" s="6"/>
       <c r="L156" s="2">
-        <v>42</v>
+        <v>16</v>
       </c>
     </row>
     <row r="157" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B157" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C157" s="2">
         <v>20260223</v>
@@ -6159,31 +6159,31 @@
         <v>11</v>
       </c>
       <c r="F157" s="2">
-        <v>125</v>
+        <v>67</v>
       </c>
       <c r="G157" s="2">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H157" s="2">
         <v>0</v>
       </c>
       <c r="I157" s="2">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="J157" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K157" s="6"/>
       <c r="L157" s="2">
-        <v>43</v>
+        <v>17</v>
       </c>
     </row>
     <row r="158" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B158" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C158" s="2">
         <v>20260223</v>
@@ -6195,23 +6195,23 @@
         <v>11</v>
       </c>
       <c r="F158" s="2">
-        <v>34</v>
+        <v>107</v>
       </c>
       <c r="G158" s="2">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="H158" s="2">
         <v>0</v>
       </c>
       <c r="I158" s="2">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="J158" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K158" s="6"/>
       <c r="L158" s="2">
-        <v>44</v>
+        <v>18</v>
       </c>
     </row>
     <row r="159" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6231,31 +6231,31 @@
         <v>11</v>
       </c>
       <c r="F159" s="2">
-        <v>98</v>
+        <v>64</v>
       </c>
       <c r="G159" s="2">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="H159" s="2">
         <v>0</v>
       </c>
       <c r="I159" s="2">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="J159" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K159" s="6"/>
       <c r="L159" s="2">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="160" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B160" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C160" s="2">
         <v>20260223</v>
@@ -6267,10 +6267,10 @@
         <v>11</v>
       </c>
       <c r="F160" s="2">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="G160" s="2">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="H160" s="2">
         <v>0</v>
@@ -6283,15 +6283,15 @@
       </c>
       <c r="K160" s="6"/>
       <c r="L160" s="2">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="161" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B161" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C161" s="2">
         <v>20260223</v>
@@ -6303,31 +6303,31 @@
         <v>11</v>
       </c>
       <c r="F161" s="2">
-        <v>107</v>
+        <v>70</v>
       </c>
       <c r="G161" s="2">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="H161" s="2">
         <v>0</v>
       </c>
       <c r="I161" s="2">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J161" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K161" s="6"/>
       <c r="L161" s="2">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="162" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B162" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C162" s="2">
         <v>20260223</v>
@@ -6339,10 +6339,10 @@
         <v>11</v>
       </c>
       <c r="F162" s="2">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="G162" s="2">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="H162" s="2">
         <v>0</v>
@@ -6355,7 +6355,7 @@
       </c>
       <c r="K162" s="6"/>
       <c r="L162" s="2">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="163" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6375,31 +6375,31 @@
         <v>11</v>
       </c>
       <c r="F163" s="2">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="G163" s="2">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="H163" s="2">
         <v>0</v>
       </c>
       <c r="I163" s="2">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="J163" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K163" s="6"/>
       <c r="L163" s="2">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="164" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B164" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C164" s="2">
         <v>20260223</v>
@@ -6411,31 +6411,31 @@
         <v>11</v>
       </c>
       <c r="F164" s="2">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="G164" s="2">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="H164" s="2">
         <v>0</v>
       </c>
       <c r="I164" s="2">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="J164" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K164" s="6"/>
       <c r="L164" s="2">
-        <v>22</v>
+        <v>36</v>
       </c>
     </row>
     <row r="165" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B165" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C165" s="2">
         <v>20260223</v>
@@ -6447,31 +6447,31 @@
         <v>11</v>
       </c>
       <c r="F165" s="2">
+        <v>67</v>
+      </c>
+      <c r="G165" s="2">
         <v>75</v>
       </c>
-      <c r="G165" s="2">
-        <v>50</v>
-      </c>
       <c r="H165" s="2">
         <v>0</v>
       </c>
       <c r="I165" s="2">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J165" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K165" s="6"/>
       <c r="L165" s="2">
-        <v>23</v>
+        <v>37</v>
       </c>
     </row>
     <row r="166" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B166" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C166" s="2">
         <v>20260223</v>
@@ -6483,23 +6483,23 @@
         <v>11</v>
       </c>
       <c r="F166" s="2">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="G166" s="2">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="H166" s="2">
         <v>0</v>
       </c>
       <c r="I166" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J166" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K166" s="6"/>
       <c r="L166" s="2">
-        <v>24</v>
+        <v>38</v>
       </c>
     </row>
     <row r="167" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6519,130 +6519,22 @@
         <v>11</v>
       </c>
       <c r="F167" s="2">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="G167" s="2">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="H167" s="2">
         <v>0</v>
       </c>
       <c r="I167" s="2">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="J167" s="5" t="b">
         <v>1</v>
       </c>
       <c r="K167" s="6"/>
       <c r="L167" s="2">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="168" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A168" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B168" s="2">
-        <v>2</v>
-      </c>
-      <c r="C168" s="2">
-        <v>20260223</v>
-      </c>
-      <c r="D168" s="1">
-        <v>5</v>
-      </c>
-      <c r="E168" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F168" s="2">
-        <v>67</v>
-      </c>
-      <c r="G168" s="2">
-        <v>75</v>
-      </c>
-      <c r="H168" s="2">
-        <v>0</v>
-      </c>
-      <c r="I168" s="2">
-        <v>33</v>
-      </c>
-      <c r="J168" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="K168" s="6"/>
-      <c r="L168" s="2">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="169" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A169" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B169" s="2">
-        <v>2</v>
-      </c>
-      <c r="C169" s="2">
-        <v>20260223</v>
-      </c>
-      <c r="D169" s="1">
-        <v>5</v>
-      </c>
-      <c r="E169" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F169" s="2">
-        <v>30</v>
-      </c>
-      <c r="G169" s="2">
-        <v>1</v>
-      </c>
-      <c r="H169" s="2">
-        <v>0</v>
-      </c>
-      <c r="I169" s="2">
-        <v>34</v>
-      </c>
-      <c r="J169" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="K169" s="6"/>
-      <c r="L169" s="2">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="170" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A170" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B170" s="2">
-        <v>2</v>
-      </c>
-      <c r="C170" s="2">
-        <v>20260223</v>
-      </c>
-      <c r="D170" s="1">
-        <v>5</v>
-      </c>
-      <c r="E170" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F170" s="2">
-        <v>52</v>
-      </c>
-      <c r="G170" s="2">
-        <v>25</v>
-      </c>
-      <c r="H170" s="2">
-        <v>0</v>
-      </c>
-      <c r="I170" s="2">
-        <v>32</v>
-      </c>
-      <c r="J170" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="K170" s="6"/>
-      <c r="L170" s="2">
         <v>39</v>
       </c>
     </row>

</xml_diff>